<commit_message>
Add Hebrew flashcards from life without books exercise
</commit_message>
<xml_diff>
--- a/etc/hebrew/adjectives.xlsx
+++ b/etc/hebrew/adjectives.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1305,6 +1305,230 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>modern</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>מוֹדֶרְנִי</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>מוֹדֶרְנִית</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>מוֹדֶרְנִיִּים</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>מוֹדֶרְנִיּוֹת</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Israeli</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>יִשְׂרְאֵלִי</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>יִשְׂרְאֵלִית</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>יִשְׂרְאֵלִים</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>יִשְׂרְאֵלִיּוֹת</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>last; recent</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>אַחֲרוֹן</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>אַחֲרוֹנָה</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>אַחֲרוֹנִים</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>אַחֲרוֹנוֹת</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>ancient</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>עַתִּיק</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>עַתִּיקָה</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>עַתִּיקִים</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>עַתִּיקוֹת</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>big; great</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>גָּדוֹל</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>גְּדוֹלָה</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>גְּדוֹלִים</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>גְּדוֹלוֹת</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Greek</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>יְוָנִי</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>יְוָנִית</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>יְוָנִים</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>יְוָנִיּוֹת</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>postmodern</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>פּוֹסְט מוֹדֶרְנִי</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>פּוֹסְט מוֹדֶרְנִית</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>פּוֹסְט מוֹדֶרְנִיִּים</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>פּוֹסְט מוֹדֶרְנִיּוֹת</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Hebrew flashcards from directions exercise
</commit_message>
<xml_diff>
--- a/etc/hebrew/adjectives.xlsx
+++ b/etc/hebrew/adjectives.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1529,6 +1529,38 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>equal; worth; equals</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>שָׁוֶה</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>שָׁוָה</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>שָׁוִים</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>שָׁווֹת</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>adjective; math operator</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Hebrew flashcards from letter exercise
</commit_message>
<xml_diff>
--- a/etc/hebrew/adjectives.xlsx
+++ b/etc/hebrew/adjectives.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1561,6 +1561,102 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>good; well</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>טוֹב</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>טוֹבָה</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>טוֹבִים</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>טוֹבוֹת</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>happy; glad</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>שָׂמֵחַ</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>שְׂמֵחָה</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>שְׂמֵחִים</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>שְׂמֵחוֹת</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>bad</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>רַע</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>רָעָה</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>רָעִים</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>רָעוֹת</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Hebrew flashcards from vocabulary exercises
</commit_message>
<xml_diff>
--- a/etc/hebrew/adjectives.xlsx
+++ b/etc/hebrew/adjectives.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1657,6 +1657,486 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>must; have to</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>חַיָּב</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>חַיֶּבֶת</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>חַיָּבִים</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>חַיָּבוֹת</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>adjective; modal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>important</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>חָשׁוּב</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>חֲשׁוּבָה</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>חֲשׁוּבִים</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>חֲשׁוּבוֹת</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>can; able</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>יָכוֹל</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>יְכוֹלָה</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>יְכוֹלִים</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>יְכוֹלוֹת</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>modal adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>פָּתוּחַ</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>פְּתוּחָה</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>פְּתוּחִים</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>פְּתוּחוֹת</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>closed</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>סָגוּר</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>סְגוּרָה</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>סְגוּרִים</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>סְגוּרוֹת</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>amazing</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>מַדְהִים</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>מַדְהִימָה</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>מַדְהִימִים</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>מַדְהִימוֹת</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>cheap</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>זוֹל</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>זוֹלָה</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>זוֹלִים</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>זוֹלוֹת</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>smart</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>חָכָם</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>חֲכָמָה</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>חֲכָמִים</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>חֲכָמוֹת</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>young</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>צָעִיר</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>צְעִירָה</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>צְעִירִים</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>צְעִירוֹת</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>hungry</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>רָעֵב</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>רְעֵבָה</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>רְעֵבִים</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>רְעֵבוֹת</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>tired</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>עָיֵף</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>עֲיֵפָה</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>עֲיֵפִים</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>עֲיֵפוֹת</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>need; should</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>צָרִיךְ</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>צְרִיכָה</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>צְרִיכִים</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>צְרִיכוֹת</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>modal adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>quiet (adj.)</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>שָׁקֵט</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>שְׁקֵטָה</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>שְׁקֵטִים</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>שְׁקֵטוֹת</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>purple</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>סָגֹול</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>סְגֻלָּה</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>סְגֻלִּים</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>סְגֻלּוֹת</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>adjective; colour</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>pink</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>וָרֹוד</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>וְרֻדָּה</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>וְרֻדִּים</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>וְרֻדּוֹת</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>adjective; colour</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Hebrew flashcards from song exercises
</commit_message>
<xml_diff>
--- a/etc/hebrew/adjectives.xlsx
+++ b/etc/hebrew/adjectives.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2137,6 +2137,102 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>beautiful</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>יָפֶה</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>יָפָה</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>יָפִים</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>יָפוֹת</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>other; another</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>אַחֵר</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>אַחֶרֶת</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>אֲחֵרִים</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>אֲחֵרוֹת</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>adjective</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>such; like this</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>כָּזֶה</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>כָּזֹאת</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>כָּאֵלֶּה</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>כָּאֵלֶּה</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>demonstrative adjective</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>